<commit_message>
Move sample-size distribution figure to Appendix B; update manuscript, data, and analysis
</commit_message>
<xml_diff>
--- a/tables_and_figures/input_tables/vars_used_by_anesrake.xlsx
+++ b/tables_and_figures/input_tables/vars_used_by_anesrake.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="22">
   <si>
     <t>Variable</t>
   </si>
@@ -70,19 +70,13 @@
     <t>Sex</t>
   </si>
   <si>
+    <t>Provided but not selected</t>
+  </si>
+  <si>
     <t>Union Membership</t>
   </si>
   <si>
-    <t>Provided but not selected</t>
-  </si>
-  <si>
     <t>Veteran Status</t>
-  </si>
-  <si>
-    <t>Voting Turnout</t>
-  </si>
-  <si>
-    <t>Voting Method</t>
   </si>
   <si>
     <t>Residence Duration</t>
@@ -428,7 +422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1">
@@ -628,10 +622,10 @@
         <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -652,18 +646,18 @@
         <v>11</v>
       </c>
       <c r="J7" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
         <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" t="s">
-        <v>19</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -724,7 +718,7 @@
         <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
         <v>11</v>
@@ -739,80 +733,16 @@
         <v>11</v>
       </c>
       <c r="G10" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="H10" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I10" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="J10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H11" t="s">
-        <v>11</v>
-      </c>
-      <c r="I11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" t="s">
-        <v>19</v>
-      </c>
-      <c r="H12" t="s">
-        <v>16</v>
-      </c>
-      <c r="I12" t="s">
-        <v>11</v>
-      </c>
-      <c r="J12" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>